<commit_message>
new customs notifiaction and new exchange rate
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
+++ b/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FA6BD9-3A27-4766-BDA6-10783C5BE16C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844AD1A6-6986-41F1-B5DF-8BE39A5D92E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="190">
   <si>
     <t>Circulars : 2024</t>
   </si>
@@ -586,6 +586,12 @@
   </si>
   <si>
     <t>Automation of Refund Application and Processing for Courier lmports through Express Cargo Clearance System (ECCS)</t>
+  </si>
+  <si>
+    <t>35/2026</t>
+  </si>
+  <si>
+    <t>SOP for clearance of imported goods through Foreign Post Offices under the Postal Import Regulations, 2025 ").</t>
   </si>
 </sst>
 </file>
@@ -623,7 +629,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -650,7 +656,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -667,7 +679,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -688,6 +700,7 @@
     <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -702,9 +715,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -985,22 +1002,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" customWidth="1"/>
     <col min="3" max="3" width="138.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="138.28515625" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="18"/>
-    </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="23"/>
+    </row>
+    <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1011,404 +1028,430 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="B7" s="22">
+        <v>46240</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="21"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B9" s="17">
         <v>46233</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="17"/>
-    </row>
-    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="D9" s="19"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="19"/>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B11" s="14">
         <v>46216</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="20"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="12"/>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="D11" s="19"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="12"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="19"/>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B13" s="11">
         <v>46214</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="19"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="10"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="B13" s="9">
-        <v>46207</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
+      <c r="D13" s="19"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="10"/>
-    </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="D14" s="19"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="9">
+        <v>46207</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D15" s="19"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="19"/>
+    </row>
+    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B17" s="9">
         <v>46206</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="19"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="D17" s="19"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="19"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>176</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B19" s="3">
         <v>46204</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="D19" s="19"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>172</v>
-      </c>
-      <c r="B19" s="3">
-        <v>46188</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>174</v>
       </c>
       <c r="B21" s="3">
         <v>46188</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>174</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46188</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>170</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B25" s="3">
         <v>46161</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C25" s="5" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>166</v>
-      </c>
-      <c r="B25" s="3">
-        <v>46156</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>168</v>
       </c>
       <c r="B27" s="3">
         <v>46156</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46156</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B31" s="3">
         <v>46149</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>165</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>162</v>
-      </c>
-      <c r="B31" s="3">
-        <v>46146</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>162</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46146</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>160</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B35" s="3">
         <v>46127</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>156</v>
-      </c>
-      <c r="B35" s="3">
-        <v>46122</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>158</v>
       </c>
       <c r="B37" s="3">
         <v>46122</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>158</v>
+      </c>
+      <c r="B39" s="3">
+        <v>46122</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>154</v>
-      </c>
-      <c r="B39" s="3">
-        <v>46113</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="B41" s="3">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>139</v>
+      </c>
+      <c r="B43" s="3">
+        <v>46112</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>141</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B45" s="3">
         <v>46111</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C45" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="47" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>142</v>
-      </c>
-      <c r="B45" s="3">
-        <v>46108</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>144</v>
       </c>
       <c r="B47" s="3">
         <v>46108</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>144</v>
+      </c>
+      <c r="B49" s="3">
+        <v>46108</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>146</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B51" s="3">
         <v>46105</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C51" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B53" s="3">
         <v>46098</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C53" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="7" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B55" s="3">
         <v>46097</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C55" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
+    <row r="57" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B57" s="3">
         <v>46091</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C57" s="5" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B57" s="3">
-        <v>46089</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="4"/>
-      <c r="B58" s="3"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B59" s="3">
+        <v>46089</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="4"/>
+      <c r="B60" s="3"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B59" s="3">
+      <c r="B61" s="3">
         <v>46081</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C61" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="63" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="B61" s="3">
-        <v>46054</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="B63" s="3">
         <v>46054</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B65" s="3">
         <v>46054</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B67" s="3">
         <v>46054</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B69" s="3">
         <v>46054</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B71" s="3">
         <v>46054</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B73" s="3">
+        <v>46054</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B75" s="3">
         <v>46037</v>
       </c>
-      <c r="C73" s="5" t="s">
+      <c r="C75" s="5" t="s">
         <v>127</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new notification of DGFT and Customs
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
+++ b/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844AD1A6-6986-41F1-B5DF-8BE39A5D92E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E99524-7001-416C-85EC-0755B498E6B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="192">
   <si>
     <t>Circulars : 2024</t>
   </si>
@@ -592,6 +592,12 @@
   </si>
   <si>
     <t>SOP for clearance of imported goods through Foreign Post Offices under the Postal Import Regulations, 2025 ").</t>
+  </si>
+  <si>
+    <t>36/2026</t>
+  </si>
+  <si>
+    <t>Return of export cargo from international waters due to closure of the Strait of Hormuz- Section 143AAof the Customs Act, 1962</t>
   </si>
 </sst>
 </file>
@@ -629,7 +635,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -638,31 +644,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
+        <fgColor rgb="FF9999FF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -679,7 +661,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -692,35 +674,24 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="15" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -728,6 +699,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF9999FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1002,22 +978,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D75"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C77"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="3" max="3" width="138.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="138.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="6.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="A1" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="23"/>
-    </row>
-    <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="16"/>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1028,430 +1004,408 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="B7" s="14">
+        <v>46254</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>188</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B9" s="3">
         <v>46240</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C9" s="5" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="21"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>186</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B11" s="3">
         <v>46233</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C11" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="D9" s="19"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="19"/>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B13" s="9">
         <v>46216</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C13" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="D11" s="19"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="19"/>
-    </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="8"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="11"/>
+    </row>
+    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>182</v>
       </c>
-      <c r="B13" s="11">
+      <c r="B15" s="12">
         <v>46214</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C15" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D13" s="19"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="19"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B17" s="3">
         <v>46207</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C17" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D15" s="19"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="19"/>
-    </row>
-    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>180</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B19" s="3">
         <v>46206</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C19" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="D17" s="19"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="19"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>176</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B21" s="3">
         <v>46204</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D19" s="19"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>172</v>
-      </c>
-      <c r="B21" s="3">
-        <v>46188</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>174</v>
       </c>
       <c r="B23" s="3">
         <v>46188</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>174</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46188</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
         <v>170</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B27" s="3">
         <v>46161</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C27" s="5" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>166</v>
-      </c>
-      <c r="B27" s="3">
-        <v>46156</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>168</v>
       </c>
       <c r="B29" s="3">
         <v>46156</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>168</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46156</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>164</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B33" s="3">
         <v>46149</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C33" s="5" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>162</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B35" s="3">
         <v>46146</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>160</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B37" s="3">
         <v>46127</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C37" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>156</v>
-      </c>
-      <c r="B37" s="3">
-        <v>46122</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>158</v>
       </c>
       <c r="B39" s="3">
         <v>46122</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>158</v>
+      </c>
+      <c r="B41" s="3">
+        <v>46122</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
         <v>154</v>
       </c>
-      <c r="B41" s="3">
+      <c r="B43" s="3">
         <v>46113</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>139</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B45" s="3">
         <v>46112</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C45" s="5" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
         <v>141</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B47" s="3">
         <v>46111</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C47" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="49" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
         <v>142</v>
-      </c>
-      <c r="B47" s="3">
-        <v>46108</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>144</v>
       </c>
       <c r="B49" s="3">
         <v>46108</v>
       </c>
       <c r="C49" s="5" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>144</v>
+      </c>
+      <c r="B51" s="3">
+        <v>46108</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>146</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B53" s="3">
         <v>46105</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C53" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B55" s="3">
         <v>46098</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C55" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="7" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B57" s="3">
         <v>46097</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C57" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+    <row r="59" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B57" s="3">
+      <c r="B59" s="3">
         <v>46091</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C59" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B59" s="3">
+      <c r="B61" s="3">
         <v>46089</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C61" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="4"/>
-      <c r="B60" s="3"/>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="4"/>
+      <c r="B62" s="3"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B61" s="3">
+      <c r="B63" s="3">
         <v>46081</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C63" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="4" t="s">
         <v>128</v>
-      </c>
-      <c r="B63" s="3">
-        <v>46054</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="4" t="s">
-        <v>129</v>
       </c>
       <c r="B65" s="3">
         <v>46054</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B67" s="3">
         <v>46054</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B69" s="3">
         <v>46054</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B71" s="3">
         <v>46054</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B73" s="3">
         <v>46054</v>
       </c>
       <c r="C73" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B75" s="3">
+        <v>46054</v>
+      </c>
+      <c r="C75" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="4" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B75" s="3">
+      <c r="B77" s="3">
         <v>46037</v>
       </c>
-      <c r="C75" s="5" t="s">
+      <c r="C77" s="5" t="s">
         <v>127</v>
       </c>
     </row>
@@ -1467,20 +1421,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71B717D5-51C8-400B-92F4-BB86799DE007}">
   <dimension ref="A1:D66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="114.28515625" style="5" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="114.33203125" style="5" customWidth="1"/>
+    <col min="4" max="4" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1491,7 +1445,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -1502,7 +1456,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1513,7 +1467,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -1524,7 +1478,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>65</v>
       </c>
@@ -1535,7 +1489,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -1546,7 +1500,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -1557,7 +1511,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1568,7 +1522,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -1579,7 +1533,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1590,7 +1544,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>77</v>
       </c>
@@ -1601,7 +1555,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1612,7 +1566,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1623,7 +1577,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>83</v>
       </c>
@@ -1634,7 +1588,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -1645,7 +1599,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>87</v>
       </c>
@@ -1656,7 +1610,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>89</v>
       </c>
@@ -1667,7 +1621,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>91</v>
       </c>
@@ -1678,7 +1632,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>93</v>
       </c>
@@ -1689,7 +1643,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>95</v>
       </c>
@@ -1700,7 +1654,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>110</v>
       </c>
@@ -1711,7 +1665,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>109</v>
       </c>
@@ -1722,7 +1676,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>111</v>
       </c>
@@ -1733,7 +1687,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>112</v>
       </c>
@@ -1744,7 +1698,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>113</v>
       </c>
@@ -1755,7 +1709,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>114</v>
       </c>
@@ -1766,7 +1720,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>115</v>
       </c>
@@ -1780,7 +1734,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>116</v>
       </c>
@@ -1791,7 +1745,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>117</v>
       </c>
@@ -1802,7 +1756,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>118</v>
       </c>
@@ -1813,7 +1767,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>119</v>
       </c>
@@ -1824,7 +1778,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>120</v>
       </c>
@@ -1843,20 +1797,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DD57242-AEC6-4DD9-AE8C-3A5671F24997}">
   <dimension ref="A1:D56"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" customWidth="1"/>
     <col min="3" max="3" width="106" style="5" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1867,7 +1821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1878,7 +1832,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1889,7 +1843,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1900,7 +1854,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1911,7 +1865,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1922,7 +1876,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1933,7 +1887,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1944,7 +1898,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1958,7 +1912,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1969,7 +1923,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1980,7 +1934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1991,7 +1945,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -2002,7 +1956,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -2013,7 +1967,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -2024,7 +1978,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>44</v>
       </c>
@@ -2035,7 +1989,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>45</v>
       </c>
@@ -2046,7 +2000,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>55</v>
       </c>
@@ -2057,7 +2011,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>54</v>
       </c>
@@ -2068,7 +2022,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>53</v>
       </c>
@@ -2079,7 +2033,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>52</v>
       </c>
@@ -2090,7 +2044,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>51</v>
       </c>
@@ -2101,7 +2055,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>50</v>
       </c>
@@ -2115,7 +2069,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
@@ -2126,7 +2080,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>48</v>
       </c>
@@ -2137,7 +2091,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>47</v>
       </c>
@@ -2148,7 +2102,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
new DGFT notification and Customs circular notification
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
+++ b/backend/PDF_DOC/CBIC/Circulars/Circulars.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E99524-7001-416C-85EC-0755B498E6B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2440E659-9715-41CC-83A0-F0C9DECCF07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="194">
   <si>
     <t>Circulars : 2024</t>
   </si>
@@ -598,6 +598,12 @@
   </si>
   <si>
     <t>Return of export cargo from international waters due to closure of the Strait of Hormuz- Section 143AAof the Customs Act, 1962</t>
+  </si>
+  <si>
+    <t>37/2026</t>
+  </si>
+  <si>
+    <t>Modalities for payment of exempted GST at the time of import of Raw Sugar actually imported under Advance Authorisation (AA) Scheme to be converted into Tariff Rate Quota (TRQ) Scheme.</t>
   </si>
 </sst>
 </file>
@@ -661,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -693,6 +699,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,22 +989,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C77"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C78"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
-    <col min="3" max="3" width="138.33203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="6.88671875" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+    <col min="3" max="3" width="138.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="16" t="s">
         <v>153</v>
       </c>
       <c r="B1" s="16"/>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1004,408 +1015,419 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="14">
+        <v>46261</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B8" s="18">
         <v>46254</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C8" s="19" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>188</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B10" s="3">
         <v>46240</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>186</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B12" s="3">
         <v>46233</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B14" s="9">
         <v>46216</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="11"/>
-    </row>
-    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="8"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="11"/>
+    </row>
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>182</v>
       </c>
-      <c r="B15" s="12">
+      <c r="B16" s="12">
         <v>46214</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>178</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B18" s="3">
         <v>46207</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>180</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B20" s="3">
         <v>46206</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>176</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B22" s="3">
         <v>46204</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>172</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B24" s="3">
         <v>46188</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C24" s="5" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>174</v>
       </c>
-      <c r="B25" s="3">
+      <c r="B26" s="3">
         <v>46188</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>170</v>
       </c>
-      <c r="B27" s="3">
+      <c r="B28" s="3">
         <v>46161</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C28" s="5" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>166</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B30" s="3">
         <v>46156</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>168</v>
       </c>
-      <c r="B31" s="3">
+      <c r="B32" s="3">
         <v>46156</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C32" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>164</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B34" s="3">
         <v>46149</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C34" s="5" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>162</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B36" s="3">
         <v>46146</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C36" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
+    <row r="38" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>160</v>
       </c>
-      <c r="B37" s="3">
+      <c r="B38" s="3">
         <v>46127</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C38" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>156</v>
       </c>
-      <c r="B39" s="3">
+      <c r="B40" s="3">
         <v>46122</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
+    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>158</v>
       </c>
-      <c r="B41" s="3">
+      <c r="B42" s="3">
         <v>46122</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C42" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>154</v>
       </c>
-      <c r="B43" s="3">
+      <c r="B44" s="3">
         <v>46113</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C44" s="5" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>139</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B46" s="3">
         <v>46112</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>141</v>
       </c>
-      <c r="B47" s="3">
+      <c r="B48" s="3">
         <v>46111</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C48" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
+    <row r="50" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>142</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B50" s="3">
         <v>46108</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C50" s="5" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>144</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B52" s="3">
         <v>46108</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C52" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>146</v>
       </c>
-      <c r="B53" s="3">
+      <c r="B54" s="3">
         <v>46105</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C54" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="4" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B55" s="3">
+      <c r="B56" s="3">
         <v>46098</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C56" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="7" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B57" s="3">
+      <c r="B58" s="3">
         <v>46097</v>
       </c>
-      <c r="C57" s="5" t="s">
+      <c r="C58" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
+    <row r="60" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B59" s="3">
+      <c r="B60" s="3">
         <v>46091</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C60" s="5" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="4" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B61" s="3">
+      <c r="B62" s="3">
         <v>46089</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C62" s="5" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="4"/>
-      <c r="B62" s="3"/>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="4" t="s">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="3"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B63" s="3">
+      <c r="B64" s="3">
         <v>46081</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="C64" s="5" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="4" t="s">
+    <row r="66" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B65" s="3">
+      <c r="B66" s="3">
         <v>46054</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C66" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B67" s="3">
+      <c r="B68" s="3">
         <v>46054</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="C68" s="5" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B69" s="3">
+      <c r="B70" s="3">
         <v>46054</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C70" s="5" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B71" s="3">
+      <c r="B72" s="3">
         <v>46054</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="C72" s="5" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A73" s="4" t="s">
+    <row r="74" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A74" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B74" s="3">
         <v>46054</v>
       </c>
-      <c r="C73" s="5" t="s">
+      <c r="C74" s="5" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="4" t="s">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B75" s="3">
+      <c r="B76" s="3">
         <v>46054</v>
       </c>
-      <c r="C75" s="5" t="s">
+      <c r="C76" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="4" t="s">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B77" s="3">
+      <c r="B78" s="3">
         <v>46037</v>
       </c>
-      <c r="C77" s="5" t="s">
+      <c r="C78" s="5" t="s">
         <v>127</v>
       </c>
     </row>
@@ -1421,20 +1443,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71B717D5-51C8-400B-92F4-BB86799DE007}">
   <dimension ref="A1:D66"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" customWidth="1"/>
-    <col min="3" max="3" width="114.33203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="29.6640625" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="114.28515625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1445,7 +1467,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>59</v>
       </c>
@@ -1456,7 +1478,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1467,7 +1489,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -1478,7 +1500,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>65</v>
       </c>
@@ -1489,7 +1511,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -1500,7 +1522,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -1511,7 +1533,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -1522,7 +1544,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -1533,7 +1555,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>75</v>
       </c>
@@ -1544,7 +1566,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>77</v>
       </c>
@@ -1555,7 +1577,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -1566,7 +1588,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>81</v>
       </c>
@@ -1577,7 +1599,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>83</v>
       </c>
@@ -1588,7 +1610,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -1599,7 +1621,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>87</v>
       </c>
@@ -1610,7 +1632,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>89</v>
       </c>
@@ -1621,7 +1643,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>91</v>
       </c>
@@ -1632,7 +1654,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>93</v>
       </c>
@@ -1643,7 +1665,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>95</v>
       </c>
@@ -1654,7 +1676,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>110</v>
       </c>
@@ -1665,7 +1687,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>109</v>
       </c>
@@ -1676,7 +1698,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>111</v>
       </c>
@@ -1687,7 +1709,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>112</v>
       </c>
@@ -1698,7 +1720,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>113</v>
       </c>
@@ -1709,7 +1731,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>114</v>
       </c>
@@ -1720,7 +1742,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>115</v>
       </c>
@@ -1734,7 +1756,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>116</v>
       </c>
@@ -1745,7 +1767,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>117</v>
       </c>
@@ -1756,7 +1778,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
         <v>118</v>
       </c>
@@ -1767,7 +1789,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
         <v>119</v>
       </c>
@@ -1778,7 +1800,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
         <v>120</v>
       </c>
@@ -1797,20 +1819,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DD57242-AEC6-4DD9-AE8C-3A5671F24997}">
   <dimension ref="A1:D56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.44140625" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
     <col min="3" max="3" width="106" style="5" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="25.8" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1821,7 +1843,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1832,7 +1854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1843,7 +1865,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1854,7 +1876,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1865,7 +1887,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1876,7 +1898,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1887,7 +1909,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1898,7 +1920,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1912,7 +1934,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1923,7 +1945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1934,7 +1956,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1945,7 +1967,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1956,7 +1978,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1967,7 +1989,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1978,7 +2000,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>44</v>
       </c>
@@ -1989,7 +2011,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>45</v>
       </c>
@@ -2000,7 +2022,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
         <v>55</v>
       </c>
@@ -2011,7 +2033,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
         <v>54</v>
       </c>
@@ -2022,7 +2044,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
         <v>53</v>
       </c>
@@ -2033,7 +2055,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
         <v>52</v>
       </c>
@@ -2044,7 +2066,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>51</v>
       </c>
@@ -2055,7 +2077,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>50</v>
       </c>
@@ -2069,7 +2091,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>49</v>
       </c>
@@ -2080,7 +2102,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>48</v>
       </c>
@@ -2091,7 +2113,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>47</v>
       </c>
@@ -2102,7 +2124,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>46</v>
       </c>

</xml_diff>